<commit_message>
Segundo teste da alocações para 150 dias
</commit_message>
<xml_diff>
--- a/alocacao/saidas_150/resumo_custos.xlsx
+++ b/alocacao/saidas_150/resumo_custos.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K5"/>
+  <dimension ref="A1:K6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -536,14 +536,14 @@
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>abastecimento_10wlim_150</t>
+          <t>abastecimento_00_150_2</t>
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>16523</v>
+        <v>16454</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>196</v>
+        <v>614</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -551,42 +551,42 @@
         </is>
       </c>
       <c r="E3" s="3" t="n">
-        <v>837883.34</v>
+        <v>834787.71</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>837883.34</v>
+        <v>834797.34</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>851803.14</v>
+        <v>909017.5</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>1.66</v>
+        <v>8.890000000000001</v>
       </c>
       <c r="I3" s="4" t="n">
         <v>0</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\entradas_150\abastecimento_10wlim_150.csv</t>
+          <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\entradas_150\abastecimento_00_150_2.csv</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\saidas_150\alocacao_abastecimento_10wlim_150</t>
+          <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\saidas_150\alocacao_abastecimento_00_150_2</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>abastecimento_full_150</t>
+          <t>abastecimento_10wlim_150</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>17421</v>
+        <v>16523</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>660</v>
+        <v>196</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -594,69 +594,112 @@
         </is>
       </c>
       <c r="E4" s="3" t="n">
-        <v>884912.76</v>
+        <v>837883.34</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>885003.4</v>
+        <v>837883.34</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>998557.75</v>
+        <v>851803.14</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>12.84</v>
+        <v>1.66</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>0.01</v>
+        <v>0</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\entradas_150\abastecimento_full_150.csv</t>
+          <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\entradas_150\abastecimento_10wlim_150.csv</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\saidas_150\alocacao_abastecimento_full_150</t>
+          <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\saidas_150\alocacao_abastecimento_10wlim_150</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
+          <t>abastecimento_full_150</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>17421</v>
+      </c>
+      <c r="C5" s="2" t="n">
+        <v>660</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="n">
+        <v>884912.76</v>
+      </c>
+      <c r="F5" s="3" t="n">
+        <v>885003.4</v>
+      </c>
+      <c r="G5" s="3" t="n">
+        <v>998557.75</v>
+      </c>
+      <c r="H5" s="4" t="n">
+        <v>12.84</v>
+      </c>
+      <c r="I5" s="4" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\entradas_150\abastecimento_full_150.csv</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\saidas_150\alocacao_abastecimento_full_150</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
           <t>abastecimento_limite_150</t>
         </is>
       </c>
-      <c r="B5" s="2" t="n">
+      <c r="B6" s="2" t="n">
         <v>16609</v>
       </c>
-      <c r="C5" s="2" t="n">
+      <c r="C6" s="2" t="n">
         <v>576</v>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D6" t="inlineStr">
         <is>
           <t>Sucesso</t>
         </is>
       </c>
-      <c r="E5" s="3" t="n">
+      <c r="E6" s="3" t="n">
         <v>842576.61</v>
       </c>
-      <c r="F5" s="3" t="n">
+      <c r="F6" s="3" t="n">
         <v>842605.48</v>
       </c>
-      <c r="G5" s="3" t="n">
+      <c r="G6" s="3" t="n">
         <v>935365.38</v>
       </c>
-      <c r="H5" s="4" t="n">
+      <c r="H6" s="4" t="n">
         <v>11.01</v>
       </c>
-      <c r="I5" s="4" t="n">
+      <c r="I6" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="J5" t="inlineStr">
+      <c r="J6" t="inlineStr">
         <is>
           <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\entradas_150\abastecimento_limite_150.csv</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr">
+      <c r="K6" t="inlineStr">
         <is>
           <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\saidas_150\alocacao_abastecimento_limite_150</t>
         </is>

</xml_diff>